<commit_message>
PLT1: equipment_mass property (equipment weights); loadTestReferenceSystem bound on lateral, plate and zone load tests
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/loadTestReferenceSystem.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/loadTestReferenceSystem.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9200" yWindow="3280" windowWidth="39400" windowHeight="24940" tabRatio="500" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="DictionaryName" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Definitions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="AssociatedElements" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="AlternateNames" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Lists" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DictionaryName" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssociatedElements" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlternateNames" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -995,7 +995,7 @@
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
@@ -1799,84 +1799,192 @@
         <f>IF(ISNA(VLOOKUP(B14,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B14" s="20" t="n"/>
+      <c r="B14" s="20" t="inlineStr">
+        <is>
+          <t>independent_reference_beam</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>//diggs:LateralLoadTest/diggs:referenceSystem</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15">
         <f>IF(ISNA(VLOOKUP(B15,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B15" s="2" t="n"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>independent_reference_beam</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>//diggs:PlateLoadTest/diggs:referenceSystem</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16">
         <f>IF(ISNA(VLOOKUP(B16,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B16" s="2" t="n"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>independent_reference_beam</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>//diggs:ZoneLoadTest/diggs:referenceSystem</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17">
         <f>IF(ISNA(VLOOKUP(B17,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B17" s="2" t="n"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>optical_survey</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>//diggs:LateralLoadTest/diggs:referenceSystem</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18">
         <f>IF(ISNA(VLOOKUP(B18,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B18" s="2" t="n"/>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>optical_survey</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>//diggs:PlateLoadTest/diggs:referenceSystem</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19">
         <f>IF(ISNA(VLOOKUP(B19,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B19" s="20" t="n"/>
+      <c r="B19" s="20" t="inlineStr">
+        <is>
+          <t>optical_survey</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>//diggs:ZoneLoadTest/diggs:referenceSystem</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20">
         <f>IF(ISNA(VLOOKUP(B20,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B20" s="20" t="n"/>
+      <c r="B20" s="20" t="inlineStr">
+        <is>
+          <t>satellite_positioning</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>//diggs:LateralLoadTest/diggs:referenceSystem</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21">
         <f>IF(ISNA(VLOOKUP(B21,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B21" s="20" t="n"/>
+      <c r="B21" s="20" t="inlineStr">
+        <is>
+          <t>satellite_positioning</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>//diggs:PlateLoadTest/diggs:referenceSystem</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22">
         <f>IF(ISNA(VLOOKUP(B22,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B22" s="20" t="n"/>
+      <c r="B22" s="20" t="inlineStr">
+        <is>
+          <t>satellite_positioning</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>//diggs:ZoneLoadTest/diggs:referenceSystem</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23">
         <f>IF(ISNA(VLOOKUP(B23,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B23" s="20" t="n"/>
+      <c r="B23" s="20" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>//diggs:LateralLoadTest/diggs:referenceSystem</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24">
         <f>IF(ISNA(VLOOKUP(B24,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B24" s="2" t="n"/>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>//diggs:PlateLoadTest/diggs:referenceSystem</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25">
         <f>IF(ISNA(VLOOKUP(B25,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B25" s="2" t="n"/>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>//diggs:ZoneLoadTest/diggs:referenceSystem</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26">

</xml_diff>